<commit_message>
found the ’ symbol does not work, did a find and delete
</commit_message>
<xml_diff>
--- a/LM/LM Verb and noun list.xlsx
+++ b/LM/LM Verb and noun list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\del13\nassp-checklist-annotator\LM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2F16983-743A-4AD1-9DB5-1F6A81C9D08C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81086000-2C55-41AE-886D-6CA4FE54DE02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20388" yWindow="0" windowWidth="20664" windowHeight="16656" firstSheet="1" activeTab="1" xr2:uid="{00155EAC-E9C1-4996-9667-4921A17D82C1}"/>
+    <workbookView xWindow="20388" yWindow="0" windowWidth="20664" windowHeight="16560" xr2:uid="{00155EAC-E9C1-4996-9667-4921A17D82C1}"/>
   </bookViews>
   <sheets>
     <sheet name="Verb" sheetId="2" r:id="rId1"/>
@@ -169,12 +169,6 @@
     <t>Change Program</t>
   </si>
   <si>
-    <t>Zero CDU’s (Specify N20 or N72)</t>
-  </si>
-  <si>
-    <t>Coarse Align CDU’s (Specify N20 or N72)</t>
-  </si>
-  <si>
     <t>Fine Align IMU</t>
   </si>
   <si>
@@ -1660,9 +1654,6 @@
     <t>Use Rotating External dV Reference Frame</t>
   </si>
   <si>
-    <t>Freeze External dV in Inertial Space and allow dV’s to Count</t>
-  </si>
-  <si>
     <t>dVX (Use 470 For Readout)</t>
   </si>
   <si>
@@ -1769,6 +1760,15 @@
   </si>
   <si>
     <t>RATE=3=10.0deg/sec</t>
+  </si>
+  <si>
+    <t>Zero CDUs (Specify N20 or N72)</t>
+  </si>
+  <si>
+    <t>Coarse Align CDUs (Specify N20 or N72)</t>
+  </si>
+  <si>
+    <t>Freeze External dV in Inertial Space and allow dVs to Count</t>
   </si>
 </sst>
 </file>
@@ -2163,15 +2163,15 @@
   <sheetData>
     <row r="1" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B1" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C1" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C2" t="s">
         <v>22</v>
@@ -2179,7 +2179,7 @@
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C3" t="s">
         <v>23</v>
@@ -2187,7 +2187,7 @@
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B4" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C4" t="s">
         <v>24</v>
@@ -2195,7 +2195,7 @@
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C5" t="s">
         <v>25</v>
@@ -2203,31 +2203,31 @@
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B6" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C6" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B7" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C7" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B8" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C8" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B9" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C9" t="s">
         <v>26</v>
@@ -2238,7 +2238,7 @@
         <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.3">
@@ -2246,7 +2246,7 @@
         <v>12</v>
       </c>
       <c r="C11" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.3">
@@ -2254,7 +2254,7 @@
         <v>13</v>
       </c>
       <c r="C12" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.3">
@@ -2262,7 +2262,7 @@
         <v>14</v>
       </c>
       <c r="C13" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.3">
@@ -2270,7 +2270,7 @@
         <v>15</v>
       </c>
       <c r="C14" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="15" spans="2:3" x14ac:dyDescent="0.3">
@@ -2278,7 +2278,7 @@
         <v>16</v>
       </c>
       <c r="C15" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.3">
@@ -2294,7 +2294,7 @@
         <v>21</v>
       </c>
       <c r="C17" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.3">
@@ -2318,7 +2318,7 @@
         <v>24</v>
       </c>
       <c r="C20" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.3">
@@ -2326,7 +2326,7 @@
         <v>25</v>
       </c>
       <c r="C21" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.3">
@@ -2406,7 +2406,7 @@
         <v>40</v>
       </c>
       <c r="C31" t="s">
-        <v>39</v>
+        <v>570</v>
       </c>
     </row>
     <row r="32" spans="2:3" x14ac:dyDescent="0.3">
@@ -2414,7 +2414,7 @@
         <v>41</v>
       </c>
       <c r="C32" t="s">
-        <v>40</v>
+        <v>571</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.3">
@@ -2422,7 +2422,7 @@
         <v>42</v>
       </c>
       <c r="C33" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.3">
@@ -2430,7 +2430,7 @@
         <v>43</v>
       </c>
       <c r="C34" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.3">
@@ -2438,7 +2438,7 @@
         <v>44</v>
       </c>
       <c r="C35" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.3">
@@ -2446,7 +2446,7 @@
         <v>47</v>
       </c>
       <c r="C36" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="37" spans="2:3" x14ac:dyDescent="0.3">
@@ -2454,7 +2454,7 @@
         <v>48</v>
       </c>
       <c r="C37" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.3">
@@ -2462,7 +2462,7 @@
         <v>49</v>
       </c>
       <c r="C38" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="39" spans="2:3" x14ac:dyDescent="0.3">
@@ -2470,7 +2470,7 @@
         <v>50</v>
       </c>
       <c r="C39" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="40" spans="2:3" x14ac:dyDescent="0.3">
@@ -2478,7 +2478,7 @@
         <v>52</v>
       </c>
       <c r="C40" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.3">
@@ -2486,7 +2486,7 @@
         <v>53</v>
       </c>
       <c r="C41" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="42" spans="2:3" x14ac:dyDescent="0.3">
@@ -2494,7 +2494,7 @@
         <v>54</v>
       </c>
       <c r="C42" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="43" spans="2:3" x14ac:dyDescent="0.3">
@@ -2502,7 +2502,7 @@
         <v>55</v>
       </c>
       <c r="C43" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="44" spans="2:3" x14ac:dyDescent="0.3">
@@ -2510,7 +2510,7 @@
         <v>56</v>
       </c>
       <c r="C44" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="45" spans="2:3" x14ac:dyDescent="0.3">
@@ -2518,7 +2518,7 @@
         <v>57</v>
       </c>
       <c r="C45" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="46" spans="2:3" x14ac:dyDescent="0.3">
@@ -2526,7 +2526,7 @@
         <v>58</v>
       </c>
       <c r="C46" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="47" spans="2:3" x14ac:dyDescent="0.3">
@@ -2534,7 +2534,7 @@
         <v>60</v>
       </c>
       <c r="C47" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="48" spans="2:3" x14ac:dyDescent="0.3">
@@ -2542,7 +2542,7 @@
         <v>61</v>
       </c>
       <c r="C48" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.3">
@@ -2550,7 +2550,7 @@
         <v>62</v>
       </c>
       <c r="C49" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="50" spans="2:3" x14ac:dyDescent="0.3">
@@ -2558,7 +2558,7 @@
         <v>63</v>
       </c>
       <c r="C50" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="51" spans="2:3" x14ac:dyDescent="0.3">
@@ -2566,7 +2566,7 @@
         <v>64</v>
       </c>
       <c r="C51" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.3">
@@ -2574,7 +2574,7 @@
         <v>65</v>
       </c>
       <c r="C52" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="53" spans="2:3" x14ac:dyDescent="0.3">
@@ -2582,7 +2582,7 @@
         <v>66</v>
       </c>
       <c r="C53" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="54" spans="2:3" x14ac:dyDescent="0.3">
@@ -2590,7 +2590,7 @@
         <v>67</v>
       </c>
       <c r="C54" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.3">
@@ -2598,7 +2598,7 @@
         <v>69</v>
       </c>
       <c r="C55" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="56" spans="2:3" x14ac:dyDescent="0.3">
@@ -2606,7 +2606,7 @@
         <v>70</v>
       </c>
       <c r="C56" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.3">
@@ -2614,7 +2614,7 @@
         <v>71</v>
       </c>
       <c r="C57" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="58" spans="2:3" x14ac:dyDescent="0.3">
@@ -2622,7 +2622,7 @@
         <v>72</v>
       </c>
       <c r="C58" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="59" spans="2:3" x14ac:dyDescent="0.3">
@@ -2630,7 +2630,7 @@
         <v>73</v>
       </c>
       <c r="C59" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.3">
@@ -2638,7 +2638,7 @@
         <v>74</v>
       </c>
       <c r="C60" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="61" spans="2:3" x14ac:dyDescent="0.3">
@@ -2646,7 +2646,7 @@
         <v>75</v>
       </c>
       <c r="C61" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="62" spans="2:3" x14ac:dyDescent="0.3">
@@ -2654,7 +2654,7 @@
         <v>76</v>
       </c>
       <c r="C62" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.3">
@@ -2662,7 +2662,7 @@
         <v>77</v>
       </c>
       <c r="C63" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="64" spans="2:3" x14ac:dyDescent="0.3">
@@ -2670,7 +2670,7 @@
         <v>78</v>
       </c>
       <c r="C64" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="65" spans="2:3" x14ac:dyDescent="0.3">
@@ -2678,7 +2678,7 @@
         <v>79</v>
       </c>
       <c r="C65" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.3">
@@ -2686,7 +2686,7 @@
         <v>80</v>
       </c>
       <c r="C66" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.3">
@@ -2694,7 +2694,7 @@
         <v>81</v>
       </c>
       <c r="C67" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="68" spans="2:3" x14ac:dyDescent="0.3">
@@ -2702,7 +2702,7 @@
         <v>82</v>
       </c>
       <c r="C68" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="69" spans="2:3" x14ac:dyDescent="0.3">
@@ -2710,7 +2710,7 @@
         <v>83</v>
       </c>
       <c r="C69" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.3">
@@ -2718,7 +2718,7 @@
         <v>85</v>
       </c>
       <c r="C70" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="71" spans="2:3" x14ac:dyDescent="0.3">
@@ -2726,7 +2726,7 @@
         <v>89</v>
       </c>
       <c r="C71" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="72" spans="2:3" x14ac:dyDescent="0.3">
@@ -2734,7 +2734,7 @@
         <v>90</v>
       </c>
       <c r="C72" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="73" spans="2:3" x14ac:dyDescent="0.3">
@@ -2742,7 +2742,7 @@
         <v>91</v>
       </c>
       <c r="C73" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="74" spans="2:3" x14ac:dyDescent="0.3">
@@ -2750,7 +2750,7 @@
         <v>92</v>
       </c>
       <c r="C74" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="75" spans="2:3" x14ac:dyDescent="0.3">
@@ -2758,7 +2758,7 @@
         <v>93</v>
       </c>
       <c r="C75" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="76" spans="2:3" x14ac:dyDescent="0.3">
@@ -2766,7 +2766,7 @@
         <v>95</v>
       </c>
       <c r="C76" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="77" spans="2:3" x14ac:dyDescent="0.3">
@@ -2774,7 +2774,7 @@
         <v>96</v>
       </c>
       <c r="C77" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="78" spans="2:3" x14ac:dyDescent="0.3">
@@ -2782,7 +2782,7 @@
         <v>97</v>
       </c>
       <c r="C78" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="79" spans="2:3" x14ac:dyDescent="0.3">
@@ -2790,7 +2790,7 @@
         <v>99</v>
       </c>
       <c r="C79" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -2811,993 +2811,993 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C1" t="s">
+        <v>288</v>
+      </c>
+      <c r="D1" t="s">
         <v>114</v>
-      </c>
-      <c r="B1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C1" t="s">
-        <v>290</v>
-      </c>
-      <c r="D1" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C4" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C5" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B6" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C6" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B7" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C7" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C8" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B9" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C9" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D9" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B10" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C10" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D10" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B11" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C11" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D11" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B12" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C12" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B13" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C13" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B14" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C14" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B15" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C15" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B16" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C16" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B17" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C17" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B18" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C18" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B19" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C19" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="D19" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B20" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C20" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="D20" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B21" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C21" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B22" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C22" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B23" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C23" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C24" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B25" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C25" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D25" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B26" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C26" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B27" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C27" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B28" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C28" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B29" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C29" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B30" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C30" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D30" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B31" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C31" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B32" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C32" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B33" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="C33" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B34" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C34" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B35" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="C35" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B36" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C36" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B37" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C37" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B38" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C38" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="D38" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B39" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C39" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D39" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B40" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C40" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="D40" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B41" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="C41" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="D41" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B42" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="C42" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B43" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C43" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B44" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C44" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B45" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C45" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B46" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C46" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B47" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C47" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B48" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="C48" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B49" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="C49" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B50" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="C50" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B51" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C51" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B52" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C52" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B53" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="C53" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B54" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C54" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B55" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C55" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B56" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C56" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D56" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B57" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C57" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D57" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B58" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C58" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B59" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C59" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B60" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C60" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B61" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C61" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B62" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C62" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="D62" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B63" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C63" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B64" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C64" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B65" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="C65" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B66" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C66" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B67" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C67" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B68" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C68" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B69" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C69" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B70" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C70" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B71" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="C71" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B72" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="C72" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B73" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="C73" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B74" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="C74" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B75" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="C75" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B76" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="C76" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B77" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C77" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B78" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C78" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B79" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C79" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B80" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C80" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B81" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C81" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B82" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="C82" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B83" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C83" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B84" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C84" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B85" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C85" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D86" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.3">
@@ -3821,15 +3821,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
@@ -3837,7 +3837,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B3" t="s">
         <v>1</v>
@@ -3896,7 +3896,7 @@
         <v>30</v>
       </c>
       <c r="B10" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
@@ -3912,7 +3912,7 @@
         <v>32</v>
       </c>
       <c r="B12" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -3920,7 +3920,7 @@
         <v>33</v>
       </c>
       <c r="B13" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
@@ -3928,7 +3928,7 @@
         <v>34</v>
       </c>
       <c r="B14" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
@@ -3936,7 +3936,7 @@
         <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
@@ -3960,7 +3960,7 @@
         <v>40</v>
       </c>
       <c r="B18" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
@@ -3968,7 +3968,7 @@
         <v>41</v>
       </c>
       <c r="B19" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
@@ -3976,7 +3976,7 @@
         <v>42</v>
       </c>
       <c r="B20" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
@@ -3984,7 +3984,7 @@
         <v>47</v>
       </c>
       <c r="B21" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
@@ -4080,7 +4080,7 @@
         <v>72</v>
       </c>
       <c r="B33" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
@@ -4088,7 +4088,7 @@
         <v>73</v>
       </c>
       <c r="B34" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
@@ -4096,7 +4096,7 @@
         <v>74</v>
       </c>
       <c r="B35" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
@@ -4104,7 +4104,7 @@
         <v>75</v>
       </c>
       <c r="B36" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
@@ -4112,7 +4112,7 @@
         <v>76</v>
       </c>
       <c r="B37" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
@@ -4120,7 +4120,7 @@
         <v>78</v>
       </c>
       <c r="B38" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
@@ -4128,7 +4128,7 @@
         <v>79</v>
       </c>
       <c r="B39" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -4149,442 +4149,442 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="C1" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C2" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C3" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C4" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C5" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>345</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>347</v>
-      </c>
       <c r="C6" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C7" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C8" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C9" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C10" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C11" t="s">
-        <v>536</v>
+        <v>572</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C12" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C13" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C14" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C15" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="C16" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C17" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C18" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C19" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C20" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C21" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C22" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="C23" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C24" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C25" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C26" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C27" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C28" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C29" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C30" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C31" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>331</v>
-      </c>
       <c r="C32" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C33" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>335</v>
-      </c>
       <c r="C34" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C35" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C36" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C37" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="C38" t="s">
         <v>339</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>331</v>
-      </c>
-      <c r="C38" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C39" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="C40" t="s">
         <v>342</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>331</v>
-      </c>
-      <c r="C40" t="s">
-        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -4608,36 +4608,36 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="B1" t="s">
+        <v>299</v>
+      </c>
+      <c r="C1" t="s">
         <v>300</v>
-      </c>
-      <c r="B1" t="s">
-        <v>301</v>
-      </c>
-      <c r="C1" t="s">
-        <v>302</v>
       </c>
       <c r="D1" s="2"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B2" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="C2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="B3" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -4645,10 +4645,10 @@
         <v>223</v>
       </c>
       <c r="B4" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C4" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -4656,10 +4656,10 @@
         <v>224</v>
       </c>
       <c r="B5" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="C5" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -4667,10 +4667,10 @@
         <v>225</v>
       </c>
       <c r="B6" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C6" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -4678,10 +4678,10 @@
         <v>226</v>
       </c>
       <c r="B7" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C7" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -4689,10 +4689,10 @@
         <v>231</v>
       </c>
       <c r="B8" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="C8" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -4700,10 +4700,10 @@
         <v>232</v>
       </c>
       <c r="B9" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C9" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -4711,10 +4711,10 @@
         <v>233</v>
       </c>
       <c r="B10" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C10" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -4722,10 +4722,10 @@
         <v>240</v>
       </c>
       <c r="B11" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C11" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -4733,10 +4733,10 @@
         <v>241</v>
       </c>
       <c r="B12" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C12" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -4744,10 +4744,10 @@
         <v>242</v>
       </c>
       <c r="B13" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C13" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -4755,10 +4755,10 @@
         <v>244</v>
       </c>
       <c r="B14" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C14" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -4766,10 +4766,10 @@
         <v>245</v>
       </c>
       <c r="B15" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C15" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -4777,10 +4777,10 @@
         <v>246</v>
       </c>
       <c r="B16" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C16" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -4788,10 +4788,10 @@
         <v>254</v>
       </c>
       <c r="B17" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="C17" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
@@ -4799,10 +4799,10 @@
         <v>260</v>
       </c>
       <c r="B18" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C18" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -4810,10 +4810,10 @@
         <v>261</v>
       </c>
       <c r="B19" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C19" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -4821,10 +4821,10 @@
         <v>262</v>
       </c>
       <c r="B20" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="C20" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -4832,10 +4832,10 @@
         <v>264</v>
       </c>
       <c r="B21" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="C21" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -4843,10 +4843,10 @@
         <v>265</v>
       </c>
       <c r="B22" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="C22" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
@@ -4854,10 +4854,10 @@
         <v>266</v>
       </c>
       <c r="B23" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C23" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
@@ -4865,10 +4865,10 @@
         <v>272</v>
       </c>
       <c r="B24" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="C24" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
@@ -4876,10 +4876,10 @@
         <v>274</v>
       </c>
       <c r="B25" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C25" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
@@ -4887,10 +4887,10 @@
         <v>275</v>
       </c>
       <c r="B26" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="C26" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
@@ -4898,10 +4898,10 @@
         <v>307</v>
       </c>
       <c r="B27" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C27" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
@@ -4909,10 +4909,10 @@
         <v>310</v>
       </c>
       <c r="B28" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="C28" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
@@ -4920,10 +4920,10 @@
         <v>312</v>
       </c>
       <c r="B29" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="C29" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
@@ -4931,10 +4931,10 @@
         <v>314</v>
       </c>
       <c r="B30" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C30" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
@@ -4942,334 +4942,334 @@
         <v>316</v>
       </c>
       <c r="B31" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="C31" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B32" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="C32" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="B33" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="C33" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="B34" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="C34" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B35" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="C35" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B36" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="C36" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="B37" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="C37" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="B38" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="C38" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="B39" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="C39" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="B40" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C40" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="B41" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="C41" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B42" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="C42" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="B43" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="C43" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="B44" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="B45" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="B46" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="C46" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="B47" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="C47" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="B48" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="C48" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="B49" t="s">
+        <v>419</v>
+      </c>
+      <c r="C49" t="s">
         <v>420</v>
-      </c>
-      <c r="B49" t="s">
-        <v>421</v>
-      </c>
-      <c r="C49" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="B50" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="C50" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="B51" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="C51" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="B52" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="C52" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="B53" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="C53" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="B54" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="C54" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="B55" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="C55" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="B56" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="C56" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="B57" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="C57" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="B58" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="C58" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="B59" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="C59" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="B60" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="C60" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="B61" t="s">
+        <v>444</v>
+      </c>
+      <c r="C61" t="s">
         <v>445</v>
-      </c>
-      <c r="B61" t="s">
-        <v>446</v>
-      </c>
-      <c r="C61" t="s">
-        <v>447</v>
       </c>
     </row>
   </sheetData>
@@ -5291,13 +5291,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="B1" t="s">
+        <v>299</v>
+      </c>
+      <c r="C1" t="s">
         <v>300</v>
-      </c>
-      <c r="B1" t="s">
-        <v>301</v>
-      </c>
-      <c r="C1" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -5305,10 +5305,10 @@
         <v>211</v>
       </c>
       <c r="B2" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="C2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -5316,10 +5316,10 @@
         <v>263</v>
       </c>
       <c r="B3" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="C3" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -5327,10 +5327,10 @@
         <v>267</v>
       </c>
       <c r="B4" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="C4" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -5338,10 +5338,10 @@
         <v>270</v>
       </c>
       <c r="B5" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C5" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -5349,10 +5349,10 @@
         <v>277</v>
       </c>
       <c r="B6" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="C6" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -5360,10 +5360,10 @@
         <v>303</v>
       </c>
       <c r="B7" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="C7" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -5371,10 +5371,10 @@
         <v>307</v>
       </c>
       <c r="B8" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="C8" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -5382,10 +5382,10 @@
         <v>310</v>
       </c>
       <c r="B9" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="C9" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -5393,10 +5393,10 @@
         <v>311</v>
       </c>
       <c r="B10" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="C10" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -5404,10 +5404,10 @@
         <v>312</v>
       </c>
       <c r="B11" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="C11" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -5415,10 +5415,10 @@
         <v>313</v>
       </c>
       <c r="B12" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="C12" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -5426,10 +5426,10 @@
         <v>315</v>
       </c>
       <c r="B13" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="C13" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -5437,10 +5437,10 @@
         <v>317</v>
       </c>
       <c r="B14" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="C14" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -5448,10 +5448,10 @@
         <v>337</v>
       </c>
       <c r="B15" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="C15" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -5459,10 +5459,10 @@
         <v>340</v>
       </c>
       <c r="B16" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="C16" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -5470,10 +5470,10 @@
         <v>341</v>
       </c>
       <c r="B17" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C17" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
@@ -5481,10 +5481,10 @@
         <v>342</v>
       </c>
       <c r="B18" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="C18" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -5492,10 +5492,10 @@
         <v>343</v>
       </c>
       <c r="B19" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="C19" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -5503,10 +5503,10 @@
         <v>344</v>
       </c>
       <c r="B20" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="C20" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -5514,10 +5514,10 @@
         <v>345</v>
       </c>
       <c r="B21" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="C21" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -5525,10 +5525,10 @@
         <v>346</v>
       </c>
       <c r="B22" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="C22" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
@@ -5536,10 +5536,10 @@
         <v>347</v>
       </c>
       <c r="B23" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="C23" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
@@ -5547,7 +5547,7 @@
         <v>357</v>
       </c>
       <c r="B24" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
@@ -5555,10 +5555,10 @@
         <v>360</v>
       </c>
       <c r="B25" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="C25" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
@@ -5566,10 +5566,10 @@
         <v>361</v>
       </c>
       <c r="B26" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="C26" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
@@ -5577,10 +5577,10 @@
         <v>362</v>
       </c>
       <c r="B27" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="C27" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
@@ -5588,10 +5588,10 @@
         <v>364</v>
       </c>
       <c r="B28" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="C28" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
@@ -5599,10 +5599,10 @@
         <v>365</v>
       </c>
       <c r="B29" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="C29" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
@@ -5610,10 +5610,10 @@
         <v>366</v>
       </c>
       <c r="B30" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="C30" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
@@ -5621,10 +5621,10 @@
         <v>367</v>
       </c>
       <c r="B31" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="C31" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
@@ -5632,10 +5632,10 @@
         <v>371</v>
       </c>
       <c r="B32" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="C32" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
@@ -5643,10 +5643,10 @@
         <v>372</v>
       </c>
       <c r="B33" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="C33" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
@@ -5654,10 +5654,10 @@
         <v>373</v>
       </c>
       <c r="B34" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="C34" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
@@ -5665,10 +5665,10 @@
         <v>402</v>
       </c>
       <c r="B35" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="C35" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
@@ -5676,10 +5676,10 @@
         <v>403</v>
       </c>
       <c r="B36" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="C36" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
@@ -5687,10 +5687,10 @@
         <v>423</v>
       </c>
       <c r="B37" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="C37" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
@@ -5698,10 +5698,10 @@
         <v>433</v>
       </c>
       <c r="B38" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="C38" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
@@ -5709,10 +5709,10 @@
         <v>440</v>
       </c>
       <c r="B39" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="C39" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
@@ -5720,10 +5720,10 @@
         <v>470</v>
       </c>
       <c r="B40" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="C40" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
@@ -5731,10 +5731,10 @@
         <v>471</v>
       </c>
       <c r="B41" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="C41" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
@@ -5742,10 +5742,10 @@
         <v>472</v>
       </c>
       <c r="B42" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="C42" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
@@ -5753,10 +5753,10 @@
         <v>477</v>
       </c>
       <c r="B43" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="C43" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
@@ -5764,10 +5764,10 @@
         <v>500</v>
       </c>
       <c r="B44" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="C44" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
@@ -5775,10 +5775,10 @@
         <v>501</v>
       </c>
       <c r="B45" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="C45" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
@@ -5786,10 +5786,10 @@
         <v>502</v>
       </c>
       <c r="B46" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="C46" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
@@ -5797,10 +5797,10 @@
         <v>612</v>
       </c>
       <c r="B47" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="C47" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
@@ -5808,10 +5808,10 @@
         <v>614</v>
       </c>
       <c r="B48" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="C48" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
     </row>
   </sheetData>
@@ -5830,103 +5830,103 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B1" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="B2" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="B3" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="B4" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="B5" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B6" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B7" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B8" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B9" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B10" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B11" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B12" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="21" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H21" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
     </row>
   </sheetData>
@@ -5950,19 +5950,19 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
+        <v>504</v>
+      </c>
+      <c r="C1" t="s">
+        <v>505</v>
+      </c>
+      <c r="D1" t="s">
         <v>506</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>507</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>508</v>
-      </c>
-      <c r="E1" t="s">
-        <v>509</v>
-      </c>
-      <c r="F1" t="s">
-        <v>510</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -5970,19 +5970,19 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="C2" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D2" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="E2" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="F2" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -5990,19 +5990,19 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="C3" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="D3" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="E3" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="F3" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -6010,13 +6010,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C4" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="F4" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -6024,10 +6024,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="F5" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
   </sheetData>

</xml_diff>